<commit_message>
Chapter Four: use Chapter One objectives and research questions, link discussion to Chapter Two
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0116ePZsFh2Yr8B4s3JdZBxN
</commit_message>
<xml_diff>
--- a/docs/chapter4_final/08_chapter/chapter_tables.xlsx
+++ b/docs/chapter4_final/08_chapter/chapter_tables.xlsx
@@ -3069,20 +3069,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table 4.18: Objectives and success criteria</t>
+          <t>Table 4.18: Objectives of Section 1.3 and their success criteria</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Objective</t>
+          <t>Objective, Chapter One wording</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3109,142 +3109,196 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>[EXACT CHAPTER ONE WORDING NEEDED] Objective 2, validation engine for SKU, quantity, customer details, pricing, duplicate orders, stock and mandatory fields</t>
+          <t>1. To design and develop a web-based order processing system that replaces manual order entry done through Excel sheets and through e-mail and WhatsApp messages.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>At least 90 percent validation accuracy</t>
+          <t>A working web-based system through which orders are entered and processed without rekeying</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Primary 87.2 percent, all errors. Secondary 93.6 percent, rule-targeted errors. Replicates 86.8 to 87.2 and 93.0 to 93.6</t>
+          <t>Built and deployed. Orders are entered in the portal, from an uploaded Excel or CSV sheet, or from a pasted message. 23 of 26 functional tests passed. CSV export of orders and webhooks are not built</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>84.0 to 89.8 and 91.0 to 95.6</t>
+          <t>not applicable</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Partly met</t>
+          <t>Met</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>[EXACT CHAPTER ONE WORDING NEEDED] Objective 3, fewer manual entry errors</t>
+          <t>2. To implement an automatic validation engine that checks SKU, quantity, customer details, pricing, duplicate orders, stock and mandatory fields, and to achieve at least 90 percent validation accuracy.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>At least 60 percent fewer manual entry errors</t>
+          <t>At least 90 percent validation accuracy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[DATA PENDING]</t>
+          <t>Primary 87.2 percent, all errors. Secondary 93.6 percent, rule-targeted errors. Replicates 86.8 to 87.2 and 93.0 to 93.6</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[DATA PENDING]</t>
+          <t>84.0 to 89.8 and 91.0 to 95.6</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partly met</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>[EXACT CHAPTER ONE WORDING NEEDED] Objective 3, mandatory fields</t>
+          <t>3. To reduce manual data-entry errors by at least 60 percent and to achieve 100 percent completion of mandatory fields.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>100 percent mandatory-field completion</t>
+          <t>At least 60 percent fewer manual entry errors</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>258 of 258 orders reaching approval, 100 percent in all three replicates</t>
+          <t>[DATA PENDING]</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>98.5 to 100.0</t>
+          <t>[DATA PENDING]</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Met</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>[EXACT CHAPTER ONE WORDING NEEDED] Objective 4, processing speed</t>
+          <t>3. As above</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>30 to 50 percent faster processing</t>
+          <t>100 percent completion of mandatory fields</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[DATA PENDING]</t>
+          <t>258 of 258 orders reaching approval, 100 percent in all three replicates</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[DATA PENDING]</t>
+          <t>98.5 to 100.0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Met</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>[EXACT CHAPTER ONE WORDING NEEDED] Objective 5, simulated orders</t>
+          <t>4. To improve order processing speed by 30 to 50 percent through digital approval, payment confirmation, fulfilment and delivery workflows.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>500 simulated orders processed</t>
+          <t>30 to 50 percent faster processing</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>500 orders in each of three replicates, 1,500 in all</t>
+          <t>[DATA PENDING]</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>[DATA PENDING]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Met</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Source: Sections 4.2 to 4.4. Accuracy judged on the primary measure with the secondary measure in support.</t>
+          <t>5. To evaluate the usability and acceptance of the system through a questionnaire and a test run of 500 simulated orders.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Test run of 500 simulated orders</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>500 orders in each of three replicates, 1,500 in all</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5. As above</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Usability and acceptance by questionnaire</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Reported in the questionnaire results, not in this technical chapter</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Reported separately</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Source: Section 1.3 and Sections 4.2 to 4.4 of this chapter. Accuracy judged on the primary measure with the secondary measure in support.</t>
         </is>
       </c>
     </row>
@@ -3593,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3624,6 +3678,11 @@
           <t>Check in Table 2.1</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Data quality dimension in Table 2.1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3646,6 +3705,11 @@
           <t>Mandatory fields</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Completeness</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3668,6 +3732,11 @@
           <t>SKU</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3690,6 +3759,11 @@
           <t>Quantity</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3712,6 +3786,11 @@
           <t>Stock</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3734,6 +3813,11 @@
           <t>Customer details</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Completeness</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3756,6 +3840,11 @@
           <t>Pricing</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Accuracy and consistency</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3778,6 +3867,11 @@
           <t>Customer details</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Completeness</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3800,6 +3894,11 @@
           <t>Duplicate orders</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Uniqueness</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3819,7 +3918,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>(none; additional check)</t>
+          <t>None, an additional check</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Chapter Four: plainer wording for the simulation's test customer profiles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0116ePZsFh2Yr8B4s3JdZBxN
</commit_message>
<xml_diff>
--- a/docs/chapter4_final/08_chapter/chapter_tables.xlsx
+++ b/docs/chapter4_final/08_chapter/chapter_tables.xlsx
@@ -3026,13 +3026,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table 4.17: Fictional customer companies used in the simulation</t>
+          <t>Table 4.17: Customer profiles used in the simulation</t>
         </is>
       </c>
     </row>
@@ -3049,15 +3049,10 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>E-mail</t>
+          <t>Region</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
@@ -3076,15 +3071,10 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>folake.adeyemi@adeyemi1.example</t>
+          <t>Ikeja</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>Ikeja</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
         <is>
           <t>26</t>
         </is>
@@ -3103,15 +3093,10 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>yusuf.adebanjo@agege13.example</t>
+          <t>Ikeja</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>Ikeja</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -3130,15 +3115,10 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>blessing.okoro@ajah14.example</t>
+          <t>Lekki-Ajah</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
-        <is>
-          <t>Lekki-Ajah</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
         <is>
           <t>25</t>
         </is>
@@ -3157,15 +3137,10 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>garba.usman@apapa20.example</t>
+          <t>Lagos Mainland</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
-        <is>
-          <t>Lagos Mainland</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
         <is>
           <t>26</t>
         </is>
@@ -3184,15 +3159,10 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>segun.olatunji@bodija16.example</t>
+          <t>Ibadan</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
-        <is>
-          <t>Ibadan</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
         <is>
           <t>42</t>
         </is>
@@ -3211,15 +3181,10 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>tolulope.ogunleye@eko6.example</t>
+          <t>Lagos Island</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
-        <is>
-          <t>Lagos Island</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
         <is>
           <t>36</t>
         </is>
@@ -3238,15 +3203,10 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ngozi.eze@greenfield7.example</t>
+          <t>Lekki-Ajah</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
-        <is>
-          <t>Lekki-Ajah</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -3265,15 +3225,10 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>fatima.sani@gwarinpa15.example</t>
+          <t>Abuja</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
-        <is>
-          <t>Abuja</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -3292,15 +3247,10 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>oluwaseun.afolabi@ibadan3.example</t>
+          <t>Ibadan</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
-        <is>
-          <t>Ibadan</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
         <is>
           <t>31</t>
         </is>
@@ -3319,15 +3269,10 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>chukwuemeka.kanu@kanu2.example</t>
+          <t>Lagos Mainland</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
-        <is>
-          <t>Lagos Mainland</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
         <is>
           <t>30</t>
         </is>
@@ -3346,15 +3291,10 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>amina.bello@lekki4.example</t>
+          <t>Lekki-Ajah</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
-        <is>
-          <t>Lekki-Ajah</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -3373,15 +3313,10 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>funmilayo.adeleke@magodo19.example</t>
+          <t>Ikeja</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
-        <is>
-          <t>Ikeja</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -3400,15 +3335,10 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>kemi.lawson@marina11.example</t>
+          <t>Lagos Island</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
-        <is>
-          <t>Lagos Island</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
         <is>
           <t>17</t>
         </is>
@@ -3427,15 +3357,10 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ibrahim.musa@northgate5.example</t>
+          <t>Abuja</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
-        <is>
-          <t>Abuja</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
         <is>
           <t>16</t>
         </is>
@@ -3454,15 +3379,10 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>babatunde.oladipo@olaade8.example</t>
+          <t>Ikeja</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
-        <is>
-          <t>Ikeja</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -3481,15 +3401,10 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>adewale.akinyemi@oyo10.example</t>
+          <t>Ibadan</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
-        <is>
-          <t>Ibadan</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -3508,15 +3423,10 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>uche.nwosu@surulere12.example</t>
+          <t>Lagos Mainland</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
-        <is>
-          <t>Lagos Mainland</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -3535,15 +3445,10 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>chiamaka.obi@victoria17.example</t>
+          <t>Lagos Island</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
-        <is>
-          <t>Lagos Island</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
         <is>
           <t>26</t>
         </is>
@@ -3562,15 +3467,10 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>emeka.okafor@yaba18.example</t>
+          <t>Lagos Mainland</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
-        <is>
-          <t>Lagos Mainland</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
         <is>
           <t>28</t>
         </is>
@@ -3589,15 +3489,10 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>hauwa.abdullahi@zuma9.example</t>
+          <t>Abuja</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
-        <is>
-          <t>Abuja</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -3606,7 +3501,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Source: replicate 1, database run 5, 03_simulation/replicate1_orders.csv. All names and contact details are fictional.</t>
+          <t>Source: test customer profiles, replicate 1, database run 5, 03_simulation/replicate1_orders.csv.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Chapter Four: report error-reduction and speed criteria as Scheduled
Removes the [DATA PENDING] placeholders. Objective 3 is Partly met on the
simulation evidence, and the manual-comparison criteria of Objectives 3 and
4 are Scheduled, with the system's own evidence reported in their place.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0116ePZsFh2Yr8B4s3JdZBxN
</commit_message>
<xml_diff>
--- a/docs/chapter4_final/08_chapter/chapter_tables.xlsx
+++ b/docs/chapter4_final/08_chapter/chapter_tables.xlsx
@@ -8485,17 +8485,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[DATA PENDING]</t>
+          <t>Every rule-targeted error was stopped in all three replicates. 40.0 to 41.7 percent of errors with no rule were flagged. Reduction against manual entry not yet measured</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[DATA PENDING]</t>
+          <t>not applicable</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Scheduled</t>
         </is>
       </c>
     </row>
@@ -8539,17 +8539,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[DATA PENDING]</t>
+          <t>Median validation time 2.34 to 22.88 ms per order across the replicates. Gain against manual handling not yet measured</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>[DATA PENDING]</t>
+          <t>not applicable</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Scheduled</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Score the manual-entry comparison and report it in Chapter Four
Two participants handled B-001 to B-040 by hand. score_manual_vs_simulation.py
scores their sheets against the answer key and compares them with Verity's
simulation outcome for the same orders, using the definitions fixed in
analyze_baseline.py. Errors reached the record in 72.5 percent of orders by
hand against 15.0 percent through Verity, a reduction of 79.3 percent.
Chapter Four gains Section 4.5.9 and Table 4.29. Objective 3 becomes Met on
indicative evidence and the speed criterion stays Scheduled, because the time
a person spends entering an order in Verity was not measured.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0116ePZsFh2Yr8B4s3JdZBxN
</commit_message>
<xml_diff>
--- a/docs/chapter4_final/08_chapter/chapter_tables.xlsx
+++ b/docs/chapter4_final/08_chapter/chapter_tables.xlsx
@@ -36,6 +36,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 4.27" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 4.28" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 4.29" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 4.30" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8387,159 +8388,159 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table 4.29: Objectives of Section 1.3 and their success criteria</t>
+          <t>Table 4.29: Manual entry and Verity on the same 40 orders</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Objective, Chapter One wording</t>
+          <t>Measure</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Criterion</t>
+          <t>Manual entry</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>95% CI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Verity</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>95% CI</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. To design and develop a web-based order processing system that replaces manual order entry done through Excel sheets and through e-mail and WhatsApp messages.</t>
+          <t>Orders with an error reaching the record</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A working web-based system through which orders are entered and processed without rekeying</t>
+          <t>29 of 40, 72.5 percent</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Built and deployed. Orders are entered in the portal, from an uploaded Excel or CSV sheet, or from a pasted message. 23 of 26 functional tests passed. CSV export of orders and webhooks are not built</t>
+          <t>57.2 to 83.9</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>6 of 40, 15.0 percent</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Met</t>
+          <t>7.1 to 29.1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. To implement an automatic validation engine that checks SKU, quantity, customer details, pricing, duplicate orders, stock and mandatory fields, and to achieve at least 90 percent validation accuracy.</t>
+          <t>Planted errors flagged</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>At least 90 percent validation accuracy</t>
+          <t>6 of 26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Primary 87.2 percent, all errors. Secondary 93.6 percent, rule-targeted errors. Replicates 86.8 to 87.2 and 93.0 to 93.6</t>
+          <t>11.0 to 42.1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>84.0 to 89.8 and 91.0 to 95.6</t>
+          <t>20 of 26</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Partly met</t>
+          <t>57.9 to 89.0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. To reduce manual data-entry errors by at least 60 percent and to achieve 100 percent completion of mandatory fields.</t>
+          <t>Rule-targeted errors flagged</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>At least 60 percent fewer manual entry errors</t>
+          <t>6 of 19</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Every rule-targeted error was stopped in all three replicates. 40.0 to 41.7 percent of errors with no rule were flagged. Reduction against manual entry not yet measured</t>
+          <t>15.4 to 54.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>19 of 19</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>83.2 to 100.0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3. As above</t>
+          <t>Errors with no rule flagged</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>100 percent completion of mandatory fields</t>
+          <t>0 of 7</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>258 of 258 orders reaching approval, 100 percent in all three replicates</t>
+          <t>0.0 to 35.4</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>98.5 to 100.0</t>
+          <t>1 of 7</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Met</t>
+          <t>2.6 to 51.3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4. To improve order processing speed by 30 to 50 percent through digital approval, payment confirmation, fulfilment and delivery workflows.</t>
+          <t>Orders with a field typed differently from the message</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>30 to 50 percent faster processing</t>
+          <t>19 of 40</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Median validation time 2.34 to 22.88 ms per order across the replicates. Gain against manual handling not yet measured</t>
+          <t>32.9 to 62.5</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -8547,70 +8548,58 @@
           <t>not applicable</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5. To evaluate the usability and acceptance of the system through a questionnaire and a test run of 500 simulated orders.</t>
+          <t>Clean orders wrongly flagged</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Test run of 500 simulated orders</t>
+          <t>0 of 14</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>500 orders in each of three replicates, 1,500 in all</t>
+          <t>0.0 to 21.5</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>not applicable</t>
+          <t>1 of 14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Met</t>
+          <t>1.3 to 31.5</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5. As above</t>
+          <t>Time per order, median and mean</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Usability and acceptance shown by the questionnaire</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>System Usability Scale mean 48.86, significantly below 68. 38.5 percent would use Verity</t>
-        </is>
-      </c>
+          <t>180 s and 246 s</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>45.35 to 52.38</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Not met</t>
-        </is>
-      </c>
+          <t>not measured for a person</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Source: Section 1.3 and Sections 4.2 to 4.5 of this chapter. Accuracy judged on the primary measure with the secondary measure in support.</t>
+          <t>Source: Entry sheets of participants P01 and P02, answer key of the comparison pack and replicate 1 of the simulation, scored with score_manual_vs_simulation.py.</t>
         </is>
       </c>
     </row>
@@ -9225,6 +9214,250 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Table 4.30: Objectives of Section 1.3 and their success criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Objective, Chapter One wording</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>95% CI</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1. To design and develop a web-based order processing system that replaces manual order entry done through Excel sheets and through e-mail and WhatsApp messages.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A working web-based system through which orders are entered and processed without rekeying</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Built and deployed. Orders are entered in the portal, from an uploaded Excel or CSV sheet, or from a pasted message. 23 of 26 functional tests passed. CSV export of orders and webhooks are not built</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2. To implement an automatic validation engine that checks SKU, quantity, customer details, pricing, duplicate orders, stock and mandatory fields, and to achieve at least 90 percent validation accuracy.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>At least 90 percent validation accuracy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Primary 87.2 percent, all errors. Secondary 93.6 percent, rule-targeted errors. Replicates 86.8 to 87.2 and 93.0 to 93.6</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>84.0 to 89.8 and 91.0 to 95.6</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Partly met</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3. To reduce manual data-entry errors by at least 60 percent and to achieve 100 percent completion of mandatory fields.</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>At least 60 percent fewer manual entry errors</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>An error reached the record in 29 of 40 orders by hand and 6 of the same 40 through Verity, a reduction of 79.3 percent. Two participants, indicative</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>57.2 to 83.9 and 7.1 to 29.1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Met, indicative</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3. As above</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>100 percent completion of mandatory fields</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>258 of 258 orders reaching approval, 100 percent in all three replicates</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>98.5 to 100.0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4. To improve order processing speed by 30 to 50 percent through digital approval, payment confirmation, fulfilment and delivery workflows.</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30 to 50 percent faster processing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Manual handling took a median of 180 s per order. Verity validates in 2.34 to 22.88 ms, but the time a person spends entering an order in Verity was not measured</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5. To evaluate the usability and acceptance of the system through a questionnaire and a test run of 500 simulated orders.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Test run of 500 simulated orders</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>500 orders in each of three replicates, 1,500 in all</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5. As above</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Usability and acceptance shown by the questionnaire</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>System Usability Scale mean 48.86, significantly below 68. 38.5 percent would use Verity</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>45.35 to 52.38</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Source: Section 1.3 and Sections 4.2 to 4.5 of this chapter. Accuracy judged on the primary measure with the secondary measure in support.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>